<commit_message>
Add one-file upload zips, clean BOMs, XLSX BOM for MacroFab
- new --step zip in build_vendor_packages.py bundles each vendor package
  (gerbers + BOM + positions + README) into <board>.zip for single-upload
- exclude board features (logos, test pads, mounting holes, net ties) from
  BOM and CPL output; verify now enforces strict BOM<->CPL designator equality
- MacroFab BOM is XLSX now (openpyxl, CSV fallback), matching PCBWay
- R73 confirmed Bourns CR0402-FX-1804GLF (ETH crystal bias); README wording
  fixed (N1/N2 are logos, not net ties); regenerated all packages + zips
</commit_message>
<xml_diff>
--- a/pcb-vendors/pcbway/ddr5-testbed/ddr5-testbed-bom.xlsx
+++ b/pcb-vendors/pcbway/ddr5-testbed/ddr5-testbed-bom.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -771,72 +771,88 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>N1</t>
+          <t>R1,R5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>antmicro_logo</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>antmicro-footprints:antmicro-logo_scaled_20mm</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+          <t>antmicro-footprints:R_0402_1005Metric</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Bourns</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>CR0402-FX-1001GLF</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.bourns.com/docs/product-datasheets/cr.pdf</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>no physical part - do not order</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>N2</t>
+          <t>R2,R4,R7,R15,R16,R17,R18,R19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>oshw_logo</t>
+          <t>0R</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>antmicro-footprints:oshw-logo</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+          <t>antmicro-footprints:R_0402_1005Metric</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ERJ2GE0R00X</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://industrial.panasonic.com/cdbs/www-data/pdf/RDA0000/AOA0000C301.pdf</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>no physical part - do not order</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>R1,R5</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>240R</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -851,12 +867,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CR0402-FX-1001GLF</t>
+          <t>CR0402-FX-2400GLF</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -869,12 +885,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>R2,R4,R7,R15,R16,R17,R18,R19</t>
+          <t>R9,R10,R11,R12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0R</t>
+          <t>220R</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -884,21 +900,21 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ERJ2GE0R00X</t>
+          <t>CR0402-FX-2200GLF</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://industrial.panasonic.com/cdbs/www-data/pdf/RDA0000/AOA0000C301.pdf</t>
+          <t>https://www.bourns.com/docs/product-datasheets/cr.pdf</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -907,12 +923,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R3,R13,R14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>240R</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -927,12 +943,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CR0402-FX-2400GLF</t>
+          <t>CR0402-FX-1002GLF</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -945,188 +961,82 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>R9,R10,R11,R12</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>220R</t>
+          <t>MT60B2G8HB-48B_A</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>antmicro-footprints:R_0402_1005Metric</t>
+          <t>antmicro-footprints:BGA-82_11x9mm_Layout13x11_P0.8mm_DDR5_MO-210-AN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Micron Technology</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CR0402-FX-2200GLF</t>
+          <t>MT60B2G8HB-48B:A</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.bourns.com/docs/product-datasheets/cr.pdf</t>
+          <t>https://www.farnell.com/datasheets/3704816.pdf</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>consign - DRAM not in JLCPCB SMT library</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>R3,R13,R14</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>TPS613221A_SOT-23-5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>antmicro-footprints:R_0402_1005Metric</t>
+          <t>antmicro-footprints:SOT-23-5</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CR0402-FX-1002GLF</t>
+          <t>TPS613221ADBVT</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.bourns.com/docs/product-datasheets/cr.pdf</t>
+          <t>https://www.ti.com/lit/ds/symlink/tps61322.pdf?ts=1679307661323&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FTPS61322%252Fpart-details%252FTPS613221ADBVT%253Futm_source%253Dgoogle%2526utm_medium%253Dcpc%2526utm_campaign%253Docb-tistore-promo-app_opn_en-cpc-storeic-google-wwe%2526utm_content%253DDevice%2526ds_k%253DTPS613221ADBVT%2526DCM%253Dyes%2526gclid%253DCjwKCAjwiOCgBhAgEiwAjv5whAbq73RvnAdgvLpW8LFuSFEla1kNqoJei2y0mTqS4-Xlc-1KWPDvLxoCIUoQAvD_BwE%2526gclsrc%253Daw.ds</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TP1,TP2,TP3</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>TP_1mm_SMD</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>antmicro-footprints:TP_SMD_1mm</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>3</v>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>no physical part - do not order</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>U1</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>MT60B2G8HB-48B_A</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>antmicro-footprints:BGA-82_11x9mm_Layout13x11_P0.8mm_DDR5_MO-210-AN</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Micron Technology</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>MT60B2G8HB-48B:A</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.farnell.com/datasheets/3704816.pdf</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>consign - DRAM not in JLCPCB SMT library</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>U2</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TPS613221A_SOT-23-5</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>antmicro-footprints:SOT-23-5</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Texas Instruments</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>TPS613221ADBVT</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.ti.com/lit/ds/symlink/tps61322.pdf?ts=1679307661323&amp;ref_url=https%253A%252F%252Fwww.ti.com%252Fproduct%252FTPS61322%252Fpart-details%252FTPS613221ADBVT%253Futm_source%253Dgoogle%2526utm_medium%253Dcpc%2526utm_campaign%253Docb-tistore-promo-app_opn_en-cpc-storeic-google-wwe%2526utm_content%253DDevice%2526ds_k%253DTPS613221ADBVT%2526DCM%253Dyes%2526gclid%253DCjwKCAjwiOCgBhAgEiwAjv5whAbq73RvnAdgvLpW8LFuSFEla1kNqoJei2y0mTqS4-Xlc-1KWPDvLxoCIUoQAvD_BwE%2526gclsrc%253Daw.ds</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>